<commit_message>
include improvements without one drive
</commit_message>
<xml_diff>
--- a/data/listado_precios_clientes.xlsx
+++ b/data/listado_precios_clientes.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="PRECIOS" sheetId="1" state="visible" r:id="rId2"/>
@@ -5306,35 +5306,35 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>207</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>2026</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>2026</v>
       </c>
     </row>

</xml_diff>